<commit_message>
chore(weekly-sync): auto-pull through 2026-07-19
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/White_Mulberry/ads_report_week21.xlsx
+++ b/data/ams_weekly_data/White_Mulberry/ads_report_week21.xlsx
@@ -4195,7 +4195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4430,117 +4430,6 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>3. WM - Desk - Manual</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Camb-SB-Multiple Asin- product collection- Reach</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>B0CPT3Q25C</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>2362</v>
-      </c>
-      <c r="E7" t="n">
-        <v>45</v>
-      </c>
-      <c r="F7" t="n">
-        <v>295.8679633333333</v>
-      </c>
-      <c r="G7" t="n">
-        <v>4237.57</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>White Mulberry</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>3. WM - Desk - Manual</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Camb-SB-Multiple Asin- product collection- Reach</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>B0DQ1NV8D2</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>2362</v>
-      </c>
-      <c r="E8" t="n">
-        <v>45</v>
-      </c>
-      <c r="F8" t="n">
-        <v>295.8679633333333</v>
-      </c>
-      <c r="G8" t="n">
-        <v>4237.57</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>White Mulberry</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>3. WM - Desk - Manual</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Camb-SB-Multiple Asin- product collection- Reach</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>B0DQ4YWSMC</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>2362</v>
-      </c>
-      <c r="E9" t="n">
-        <v>45</v>
-      </c>
-      <c r="F9" t="n">
-        <v>295.8679633333333</v>
-      </c>
-      <c r="G9" t="n">
-        <v>4237.57</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>White Mulberry</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>